<commit_message>
CFO-5 y CFO-6, de la ronda 3: Áurea toma la moneda del extracto cuando la configuración no la dice, y cada extracto del material la trae; Tomás recibe en record_issues el escrito de proyecciones o actas que la ficha no cita, y puede anotarlo en reviewed con su motivo; el PDF del extracto con el ancho de cada columna
</commit_message>
<xml_diff>
--- a/tests/criterio-cfo/material/banca-pe/finanzas/20710000019-banco-ribera/2026-09/20-bancos/andino-7101/extracto.xlsx
+++ b/tests/criterio-cfo/material/banca-pe/finanzas/20710000019-banco-ribera/2026-09/20-bancos/andino-7101/extracto.xlsx
@@ -62,6 +62,11 @@
           <t>saldo</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>moneda</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
@@ -83,6 +88,11 @@
       <c r="E2">
         <v>-17280.00</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
@@ -104,6 +114,11 @@
       <c r="E3">
         <v>25200.00</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
@@ -125,6 +140,11 @@
       <c r="E4">
         <v>38200.00</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
@@ -146,6 +166,11 @@
       <c r="E5">
         <v>78320.00</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
@@ -167,6 +192,11 @@
       <c r="E6">
         <v>97200.00</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
@@ -188,6 +218,11 @@
       <c r="E7">
         <v>91200.00</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
@@ -209,6 +244,11 @@
       <c r="E8">
         <v>74916.00</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
@@ -230,6 +270,11 @@
       <c r="E9">
         <v>64916.00</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
@@ -251,6 +296,11 @@
       <c r="E10">
         <v>86156.00</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
@@ -272,6 +322,11 @@
       <c r="E11">
         <v>78156.00</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
@@ -293,6 +348,11 @@
       <c r="E12">
         <v>68999.20</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
@@ -314,6 +374,11 @@
       <c r="E13">
         <v>87879.20</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
@@ -335,6 +400,11 @@
       <c r="E14">
         <v>118559.20</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
@@ -356,6 +426,11 @@
       <c r="E15">
         <v>18559.20</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
@@ -377,6 +452,11 @@
       <c r="E16">
         <v>16959.20</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>